<commit_message>
now working fine until now still have to change backend side of token exchange
</commit_message>
<xml_diff>
--- a/doc_processor/app/leads/ed236868-e589-4eb6-974c-e442d5b7a940.xlsx
+++ b/doc_processor/app/leads/ed236868-e589-4eb6-974c-e442d5b7a940.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -643,10 +643,37 @@
           <t>muhammed.risshad@gmail.com</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>f2a1f857-2b75-49ab-824a-f0d75886d2e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-11T07:43:57.460816+00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>who is our prime minister</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>rishad</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>muhammed.risshad@gmail.com</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>28edcb00-b331-4623-95dc-e875ad964170</t>
         </is>
       </c>
     </row>

</xml_diff>